<commit_message>
mise en forme tableau protocoles de test
</commit_message>
<xml_diff>
--- a/Jeux de tests/Protocoles de tests.xlsx
+++ b/Jeux de tests/Protocoles de tests.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ProjAP\Nouveau dossier\GSB-Frais-App\Jeux de tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3762F9D2-35CC-4154-AFD9-3BA17C001EDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED27DCE9-9763-457E-87B4-338BC334EFF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D4AC787B-8E68-4DB0-B129-74856AC1034E}"/>
+    <workbookView xWindow="3075" yWindow="3075" windowWidth="21600" windowHeight="11295" xr2:uid="{D4AC787B-8E68-4DB0-B129-74856AC1034E}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,6 +36,65 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="18">
+  <si>
+    <t>Tests de connexion</t>
+  </si>
+  <si>
+    <t>Cas</t>
+  </si>
+  <si>
+    <t>Identifiant</t>
+  </si>
+  <si>
+    <t>Mot de passe</t>
+  </si>
+  <si>
+    <t>Resultat attendu</t>
+  </si>
+  <si>
+    <t>Résultat final</t>
+  </si>
+  <si>
+    <t>Prérequis</t>
+  </si>
+  <si>
+    <t>visiteur123</t>
+  </si>
+  <si>
+    <t>visiteur1</t>
+  </si>
+  <si>
+    <t>comptable1</t>
+  </si>
+  <si>
+    <t>comptable123</t>
+  </si>
+  <si>
+    <t>admin1</t>
+  </si>
+  <si>
+    <t>admin123</t>
+  </si>
+  <si>
+    <t>aucun compte</t>
+  </si>
+  <si>
+    <t>Connexion échouée</t>
+  </si>
+  <si>
+    <t>compte créé</t>
+  </si>
+  <si>
+    <t>visiteur 1</t>
+  </si>
+  <si>
+    <t>visiteur 123</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
@@ -47,12 +106,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -67,8 +132,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -383,9 +454,272 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87B6A4CA-E6E3-496F-ABF8-49A38AEF8AC7}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="2" width="17.7109375" customWidth="1"/>
+    <col min="3" max="3" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="17.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" s="2"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" s="2"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="2"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>4</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>6</v>
+      </c>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>7</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <v>8</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>9</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
+        <v>10</v>
+      </c>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>11</v>
+      </c>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
+        <v>12</v>
+      </c>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <v>13</v>
+      </c>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <v>14</v>
+      </c>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
+        <v>15</v>
+      </c>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="2">
+        <v>16</v>
+      </c>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="2">
+        <v>17</v>
+      </c>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="2">
+        <v>18</v>
+      </c>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>